<commit_message>
actualizacion documentos planificacion lab019-021
</commit_message>
<xml_diff>
--- a/fermentation_model/docs/planning/planificacion_LAB019_021_replica_lote2_2026.xlsx
+++ b/fermentation_model/docs/planning/planificacion_LAB019_021_replica_lote2_2026.xlsx
@@ -20,11 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="dd/mm/yyyy hh:mm"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy hh:mm"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -100,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -128,10 +127,16 @@
     <xf numFmtId="165" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -506,16 +511,16 @@
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="43" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Planificación LAB019-021 — Réplica del Lote 2 (LAB004-006), vendimia 2026</t>
+          <t>Planificación LAB019-021 — Réplica de LAB004 · LAB006 · LAB009, vendimia 2026</t>
         </is>
       </c>
     </row>
@@ -532,7 +537,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
+    <row r="5" ht="86" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Objetivo</t>
@@ -540,11 +545,11 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Replicar el lote LAB004-006 (mosto natural, Protocolos A y C) con el sistema de CO2 correctamente conectado y sin fugas, reproduciendo perfiles de temperatura y nutrición originales</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="54" customHeight="1">
+          <t>Replicar con el sistema de CO2 correctamente conectado y sin fugas tres fermentaciones históricas sobre el mismo diseño: LAB004 (Protocolo A) y LAB006 (Protocolo C) del 06/04, y LAB009 (Protocolo A) del 17/04, reproduciendo perfiles de temperatura y nutrición originales</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Motivo</t>
@@ -552,7 +557,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>En LAB004-006 (abril 2026) la implementación de CO2 tuvo fugas/perfil no confiable; esta réplica busca datos CO2 confiables sobre el mismo diseño experimental</t>
+          <t>En abril 2026 la medición de CO2 tuvo fugas/perfil no confiable (LAB004-006, LAB009); esta réplica busca datos CO2 confiables + trayectoria del CO2 disuelto (Carbodoseur) para observar el pool del modelo</t>
         </is>
       </c>
     </row>
@@ -564,11 +569,11 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>LAB019 = R-2L-01 (F1), Protocolo A, réplica de LAB004 · LAB020 = R-2L-02 (F2), Protocolo A, réplica de LAB005 · LAB021 = R-2L-03 (F3), Protocolo C, réplica de LAB006</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="38" customHeight="1">
+          <t>LAB019 = R-2L-01 (F1), Protocolo A, réplica de LAB004 · LAB020 = R-2L-02 (F2), Protocolo C, réplica de LAB006 · LAB021 = R-2L-03 (F3), Protocolo A, réplica de LAB009 (grupo 17/04, sin registro Maestro)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Medio y cepa</t>
@@ -576,7 +581,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Mosto natural Sauvignon blanc; Saccharomyces cerevisiae Zymaflore X5; 2 L por reactor</t>
+          <t>Mosto natural Sauvignon blanc; Saccharomyces cerevisiae Zymaflore X5; 2 L por reactor; 1 g de levadura + Springferm Xtrem 1.00 g + FDA 0.40 g en la inoculación</t>
         </is>
       </c>
     </row>
@@ -612,7 +617,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Seca (GF&lt;4 g/L) entre t=122-146 h (sáb 26-dom 27/09); fin del protocolo t=163 h ≈ 6.8 días</t>
+          <t>Seca (GF&lt;4 g/L) entre t=120-146 h (sáb 16:00-dom 18:00); fin del protocolo t=160-171 h ≈ 6.7-7.1 días</t>
         </is>
       </c>
     </row>
@@ -624,7 +629,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Seca entre t=170-194 h (lun 28-mar 29/09); fin del protocolo t=211 h ≈ 8.8 días</t>
+          <t>Seca entre t=170-194 h (lun 28/09 18:00 - mar 29/09 18:00); fin del protocolo t=219 h ≈ 9.1 días</t>
         </is>
       </c>
     </row>
@@ -636,11 +641,11 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Jueves 01/10/2026: muestra condicional de LAB021, desmontaje y cierre</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="102" customHeight="1">
+          <t>Jueves 01/10/2026: muestra condicional de F2 (LAB020), vaciado y cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="86" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Muestras planificadas</t>
@@ -648,7 +653,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>17 eventos (PI + 15 + mini -02B; -15 condicional), 3 reactores por evento. Visitas completas 08:30 y 14:30 (viernes solo 08:30) + mini-muestreo martes 11:45 (solo Carbodoseur + densidad/Brix/DO); Cada visita demora ~1.5-2 h de procesamiento (3 fermentadores × Y15, Oculyze, Carbodoseur, Brix, densidad, DO)</t>
+          <t>22 eventos (PI + 21; -21 condicional), 3 reactores por evento. Visitas completas 08:30 y 14:30 + mini-muestreos 11:15/16:40 (mar-jue) y 11:00 (vie); Cada visita demora ~1.5-2 h de procesamiento (3 fermentadores × Y15, Oculyze, Carbodoseur, Brix, densidad, DO)</t>
         </is>
       </c>
     </row>
@@ -660,7 +665,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>8 eventos fijos (PI, -01, -02, -02B, -05, -06, -09, -14) + -15 si se toma; ~100 mL por lectura (≈0.8-0.9 L/reactor). Motivo: observar el pool de CO2 disuelto — IC real (≠0), trayectoria pre/post onset (threshold vs continuous release) y validación de Csat(T)</t>
+          <t>11 lecturas fijas + 1 condicional (~100 mL c/u; la alícuota se devuelve al reactor): PI y t0 (IC real ≠0), 4 puntos del martes (16.5/19.25/22.5/24.7 h: trayectoria del onset, discrimina threshold vs continuous), meseta y pre-pulso (mié), post-pulso (jue y vie) y post-cambios T (lun 28)</t>
         </is>
       </c>
     </row>
@@ -672,7 +677,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Lun-jue 8:00-17:30: visitas de muestreo 08:30 (proceso hasta ~10:30) y 14:30 (hasta ~16:30); almuerzo 13:00-14:30; limpieza desde 17:00. Viernes 8:00-12:30 (visita 08:30). Fin de semana sin personal</t>
+          <t>Lun-jue 8:00-17:30: visitas 08:30 y 14:30 + minis 11:15/16:40 (cada visita completa ~1.5-2 h de proceso); almuerzo 13:00-14:30; limpieza desde 17:00. Viernes 8:00-12:30. Fin de semana sin personal</t>
         </is>
       </c>
     </row>
@@ -716,7 +721,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="38" customHeight="1">
+    <row r="20" ht="22" customHeight="1">
       <c r="B20" s="3" t="inlineStr">
         <is>
           <t>LAB019</t>
@@ -734,7 +739,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>LAB004</t>
+          <t>LAB004 (06/04)</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -748,7 +753,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="38" customHeight="1">
+    <row r="21" ht="22" customHeight="1">
       <c r="B21" s="4" t="inlineStr">
         <is>
           <t>LAB020</t>
@@ -761,22 +766,22 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>LAB005</t>
+          <t>LAB006 (06/04)</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>18 °C → 21 °C (t=99 h) → 16 °C (t=171 h)</t>
+          <t>16 °C → 18 °C (t=123 h) → 21 °C (t=219 h)</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>t=51 h (densidad 1040)</t>
+          <t>t=75 h (densidad 1040)</t>
         </is>
       </c>
     </row>
@@ -793,22 +798,22 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>LAB006</t>
+          <t>LAB009 (17/04)</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>16 °C → 18 °C (t=123 h) → 21 °C (t=219 h)</t>
+          <t>18 °C → 21 °C (t=96 h) → 16 °C (t=168 h, inferido)</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>t=75 h (densidad 1040)</t>
+          <t>t=48 h (vía ICS; sin registro en workbook)</t>
         </is>
       </c>
     </row>
@@ -834,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I44"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -842,7 +847,7 @@
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="58" customWidth="1" min="9" max="9"/>
@@ -1115,7 +1120,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
+    <row r="11" ht="38" customHeight="1">
       <c r="B11" s="7" t="n">
         <v>46286</v>
       </c>
@@ -1301,7 +1306,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="54" customHeight="1">
+    <row r="16" ht="38" customHeight="1">
       <c r="B16" s="8" t="n">
         <v>46287</v>
       </c>
@@ -1320,7 +1325,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>MUESTRA -02 (t=16.5 h) + Carbodoseur</t>
+          <t>MUESTRA 02 02 (t=16.5 h) + Carbodoseur</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1335,11 +1340,11 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Fase de latencia/adaptación (CO2 detectable desde ~8-10 h). Ventana de onset: discrimina acumulación previa (threshold) vs emisión temprana (continuous)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="70" customHeight="1">
+          <t>Pre-onset. Inicio de la trayectoria del pool del martes (16.5 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
       <c r="B17" s="7" t="n">
         <v>46287</v>
       </c>
@@ -1350,15 +1355,15 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>19.75</v>
+        <v>19.25</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>MINI-MUESTRA -02B (t=19.75 h) + Carbodoseur</t>
+          <t>MINI-MUESTRA 03 (t=19.25 h) + Carbodoseur</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1373,11 +1378,11 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Punto intermedio de la trayectoria del pool pre-onset: día martes queda 16.5 / 19.75 / 22.5 h. ~15-20 min; no interfiere con el almuerzo ni la visita de las 14:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
+          <t>Mini-muestreo (~15-20 min): trayectoria del pool pre-onset (19.25 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="54" customHeight="1">
       <c r="B18" s="8" t="n">
         <v>46287</v>
       </c>
@@ -1396,7 +1401,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>MUESTRA -03 (t=22.5 h)</t>
+          <t>MUESTRA 04 04 (t=22.5 h) + Carbodoseur</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1411,30 +1416,30 @@
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Inicio de fase exponencial</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="38" customHeight="1">
+          <t>Borde del onset esperado de A (referencias: 24-30 h según loggers de abril; 22-24 h en LAB016-018 a 20 °C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
       <c r="B19" s="7" t="n">
-        <v>46288</v>
+        <v>46287</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>martes</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>40.5</v>
+        <v>24.67</v>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>MUESTRA -04 (t=40.5 h)</t>
+          <t>MINI-MUESTRA 05 (t=24.67 h) + Carbodoseur</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -1449,11 +1454,11 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Crecimiento exponencial; previo al pulso 2 de A (mié 19:00)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="54" customHeight="1">
+          <t>En/frontera del onset de A (~24.7 h): el punto que discrimina acumulación previa (threshold) vs emisión temprana (continuous)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
       <c r="B20" s="8" t="n">
         <v>46288</v>
       </c>
@@ -1464,15 +1469,15 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="E20" s="10" t="n">
-        <v>46.5</v>
+        <v>40.5</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>MUESTRA -05 (t=46.5 h) + Carbodoseur</t>
+          <t>MUESTRA 06 06 (t=40.5 h) + Carbodoseur</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1487,7 +1492,7 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Última muestra antes del pulso 2 de A (19:00). Meseta exponencial: nivel del pool vs Csat. Contingencia: densidad esperada ~1044 g/L (LAB004 t=50 h)</t>
+          <t>Meseta exponencial: nivel del pool vs Csat</t>
         </is>
       </c>
     </row>
@@ -1502,53 +1507,53 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="E21" s="9" t="n">
-        <v>51</v>
+        <v>43.25</v>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>Pulso nutricional 2 — condición A</t>
+          <t>MINI-MUESTRA 07 (t=43.25 h)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>F1,F2</t>
+          <t>F1,F2,F3</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Automático</t>
+          <t>Muestreo</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Springferm Xtrem 1.00 g + FDA 0.40 g por reactor (t=51 h; original: densidad 1040)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="38" customHeight="1">
+          <t>Mini-muestreo de densidad (vigilar cruce de 1040 para los pulsos de la tarde)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="70" customHeight="1">
       <c r="B22" s="8" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="E22" s="10" t="n">
-        <v>64.5</v>
+        <v>46.5</v>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>MUESTRA -06 (t=64.5 h) + Carbodoseur</t>
+          <t>MUESTRA 08 08 (t=46.5 h) + Carbodoseur</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1563,68 +1568,68 @@
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>13.5 h post-pulso A: respuesta del pool al pulso. Verificar en el log que la bomba ejecutó el pulso</t>
+          <t>Pre-pulso 2: F3 pulsa a las 16:00 (t=48) y F1 a las 19:00 (t=51). Contingencia densidad F1: esperada ~1044 g/L (LAB004 t=50); si ≥1052 reprogramar a jue 08:30; si ≤1036 adelantar a mié 18:00</t>
         </is>
       </c>
     </row>
     <row r="23" ht="38" customHeight="1">
       <c r="B23" s="7" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="E23" s="9" t="n">
-        <v>64.5</v>
+        <v>48</v>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>Verificar log: pulso 2 de A ejecutado</t>
+          <t>Pulso nutricional 2 — F3 (réplica de LAB009)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>F1,F2</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Verificación</t>
+          <t>Automático</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>Revisar flanco de la bomba en el logger (análogo a nutricion_activa de LAB016-018)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="54" customHeight="1">
+          <t>Springferm Xtrem 1.00 g + FDA 0.40 g (t=48 h, vía ICS del original). Llegando de la visita de las 14:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
       <c r="B24" s="8" t="n">
-        <v>46289</v>
+        <v>46288</v>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="E24" s="10" t="n">
-        <v>70.5</v>
+        <v>48.67</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>MUESTRA -07 (t=70.5 h)</t>
+          <t>MINI-MUESTRA 09 (t=48.67 h)</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1639,281 +1644,283 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>Última muestra antes del pulso 2 de C (jue 19:00). Contingencia: densidad esperada ~1040 g/L (LAB006 t=74 h)</t>
+          <t>2.7 h post-pulso de F3 / pre-pulso de F1 (19:00): contraste entre fermentadores en la misma visita</t>
         </is>
       </c>
     </row>
     <row r="25" ht="38" customHeight="1">
       <c r="B25" s="7" t="n">
+        <v>46288</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>miércoles</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>51</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Pulso nutricional 2 — F1 (réplica de LAB004)</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Springferm Xtrem 1.00 g + FDA 0.40 g (t=51 h; original: densidad 1040)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="B26" s="8" t="n">
         <v>46289</v>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>jueves</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>MUESTRA 10 10 (t=64.5 h) + Carbodoseur</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Muestreo</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Post-pulso: F1 a 13.5 h y F3 a 16.5 h del suyo; F2 pre-pulso (75 h = jue 19:00). Verificar logs de bomba del miércoles</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="B27" s="7" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>jueves</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>64.5</v>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Verificar log: pulsos 2 de F3 y F1 ejecutados</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>F3,F1</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Verificación</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Revisar flancos de la bomba en el logger (análogo a nutricion_activa de LAB016-018)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="B28" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>jueves</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>67.25</v>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>MINI-MUESTRA 11 (t=67.25 h)</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Muestreo</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>Mini-muestreo de densidad (cruce de 1040 de F2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="70" customHeight="1">
+      <c r="B29" s="7" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>jueves</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>MUESTRA 12 12 (t=70.5 h)</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Muestreo</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>Última muestra antes del pulso 2 de F2 (19:00). Contingencia densidad: esperada ~1040 g/L (LAB006 t=74); si ≥1048 reprogramar a vie 08:30; si ≤1032 adelantar a jue 18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="8" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>jueves</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>72.67</v>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>MINI-MUESTRA 13 (t=72.67 h)</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Muestreo</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>2.7 h pre-pulso de F2 (19:00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="38" customHeight="1">
+      <c r="B31" s="7" t="n">
+        <v>46289</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>jueves</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E31" s="9" t="n">
         <v>75</v>
       </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>Pulso nutricional 2 — condición C</t>
-        </is>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Pulso nutricional 2 — F2 (réplica de LAB006)</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>Automático</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>Springferm Xtrem 1.00 g + FDA 0.40 g (t=75 h; original: densidad 1040)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="38" customHeight="1">
-      <c r="B26" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>viernes</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>MUESTRA -08 (t=88.5 h)</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>F1,F2,F3</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Muestreo</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>13.5 h post-pulso C; cierre de semana (salida viernes 12:30)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="B27" s="7" t="n">
-        <v>46290</v>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>viernes</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Verificar log: pulso 2 de C ejecutado</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Verificación</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>Ídem</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="54" customHeight="1">
-      <c r="B28" s="8" t="n">
-        <v>46290</v>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>viernes</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="n">
-        <v>91.5</v>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Cierre de fin de semana</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>F1,F2,F3</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Verificación</t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>Confirmar programación del setpoint F3 (sáb 19:00), capacidad de loggers hasta el lunes y bombas sin eventos pendientes; 12:00-12:30 limpieza y salida</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="7" t="n">
-        <v>46290</v>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>viernes</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>99</v>
-      </c>
-      <c r="F29" s="3" t="inlineStr">
-        <is>
-          <t>Setpoint 21 °C (A)</t>
-        </is>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>F1,F2</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
-      </c>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>t=99 h (réplica exacta del original)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="86" customHeight="1">
-      <c r="B30" s="8" t="n">
-        <v>46291</v>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>sábado</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>Fin de semana sin personal</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>F1,F2,F3</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>Sin personal</t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>Sábado y domingo: logging continuo CO2/T; único evento: setpoint F3 18 °C (sáb 19:00, automático). Ventana ciega de muestreo: la sequedad de A (t=122-146 h) ocurrirá aquí; el CO2 continuo sin fugas cubre el intervalo</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="B31" s="7" t="n">
-        <v>46291</v>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>sábado</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="E31" s="9" t="n">
-        <v>123</v>
-      </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t>Setpoint 18 °C (C)</t>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
-      </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>t=123 h (réplica exacta del original)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="54" customHeight="1">
       <c r="B32" s="8" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1922,11 +1929,11 @@
         </is>
       </c>
       <c r="E32" s="10" t="n">
-        <v>160.5</v>
+        <v>88.5</v>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>MUESTRA -09 (t=160.5 h) + Carbodoseur</t>
+          <t>MUESTRA 14 14 (t=88.5 h) + Carbodoseur</t>
         </is>
       </c>
       <c r="G32" s="4" t="inlineStr">
@@ -1941,17 +1948,17 @@
       </c>
       <c r="I32" s="4" t="inlineStr">
         <is>
-          <t>Post-fin de semana: A seca esperada (t=122-146 h). Post-cambios T (A 21 °C, C 18 °C): valida Csat(T). Descargar/respaldar datos</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="38" customHeight="1">
+          <t>Post-pulso de F2 (13.5 h) + A tardía. Verificar log del pulso de F2 y del cambio T de F3 (vie 16:00); F1 cambia a 21 °C hoy 19:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
       <c r="B33" s="7" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -1960,16 +1967,16 @@
         </is>
       </c>
       <c r="E33" s="9" t="n">
-        <v>160.5</v>
+        <v>88.5</v>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>Verificar cambios T del finde + respaldo</t>
+          <t>Verificar log: pulso 2 de F2 ejecutado</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>F1,F2,F3</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
@@ -1979,30 +1986,30 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Confirmar setpoint 21 °C en F1/F2 (vie 19:00) y 18 °C en F3 (sáb 19:00); descargar y respaldar datos</t>
+          <t>Ídem</t>
         </is>
       </c>
     </row>
     <row r="34" ht="38" customHeight="1">
       <c r="B34" s="8" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E34" s="10" t="n">
-        <v>166.5</v>
+        <v>91</v>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>MUESTRA -10 (t=166.5 h)</t>
+          <t>MINI-MUESTRA 15 (t=91 h)</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
@@ -2017,387 +2024,651 @@
       </c>
       <c r="I34" s="4" t="inlineStr">
         <is>
-          <t>Confirmación de sequedad A (GF&lt;2 g/L en 2 muestras seguidas da por terminados LAB019/020)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="22" customHeight="1">
+          <t>Última del día antes del cambio T de F1 (19:00); cierre de semana (salida 12:30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="70" customHeight="1">
       <c r="B35" s="7" t="n">
-        <v>46293</v>
+        <v>46290</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Cierre de fin de semana</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>Verificación</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar setpoint F3 21 °C ejecutado (16:00) y F1 21 °C programado (19:00); F2 cambia el sábado 19:00; capacidad de loggers hasta el lunes; 12:00-12:30 limpieza y salida</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="38" customHeight="1">
+      <c r="B36" s="8" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>viernes</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="n">
+        <v>96</v>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Setpoint 21 °C — F3</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>t=96 h (réplica exacta del original, ejecutado con personal presente)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="B37" s="7" t="n">
+        <v>46290</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>viernes</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="E35" s="9" t="n">
-        <v>171</v>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>Setpoint 16 °C (A)</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>F1,F2</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="E37" s="9" t="n">
+        <v>99</v>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Setpoint 21 °C — F1</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>Automático</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>t=171 h (réplica exacta del original)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="B36" s="8" t="n">
-        <v>46294</v>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>martes</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>08:30</t>
-        </is>
-      </c>
-      <c r="E36" s="10" t="n">
-        <v>184.5</v>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>MUESTRA -11 (t=184.5 h)</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>t=99 h (réplica exacta del original, sin personal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="86" customHeight="1">
+      <c r="B38" s="8" t="n">
+        <v>46291</v>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>sábado</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="n"/>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Fin de semana sin personal</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
         <is>
           <t>F1,F2,F3</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>Muestreo</t>
-        </is>
-      </c>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>Muestra final de A (condicional); C en fase final</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="38" customHeight="1">
-      <c r="B37" s="7" t="n">
-        <v>46294</v>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>martes</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="E37" s="9" t="n">
-        <v>190.5</v>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>MUESTRA -12 (t=190.5 h)</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>F1,F2,F3</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Muestreo</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>Cercanía a sequedad de C (LAB006: GF=4.7 g/L a t=170 h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="38" customHeight="1">
-      <c r="B38" s="8" t="n">
-        <v>46294</v>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>martes</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="E38" s="10" t="n">
-        <v>190.5</v>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Si LAB019/020 confirmadas secas: vaciar F1/F2</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>F1,F2</t>
-        </is>
-      </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Cierre</t>
+          <t>Sin personal</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
         <is>
-          <t>Criterio: GF&lt;2 g/L en 2 muestras consecutivas (-09/-10)</t>
+          <t>Sábado y domingo: logging continuo CO2/T; únicos eventos: setpoint F2 18 °C (sáb 19:00, automático). Ventana ciega de muestreo: la sequedad de A (t=120-146 h) ocurrirá aquí; el CO2 continuo sin fugas cubre el intervalo</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="B39" s="7" t="n">
-        <v>46295</v>
+        <v>46291</v>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>sábado</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="n">
+        <v>123</v>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Setpoint 18 °C — F2</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>t=123 h (réplica exacta del original, sin personal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="54" customHeight="1">
+      <c r="B40" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>lunes</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="E39" s="9" t="n">
-        <v>208.5</v>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>MUESTRA -13 (t=208.5 h)</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="E40" s="10" t="n">
+        <v>160.5</v>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>MUESTRA 16 16 (t=160.5 h) + Carbodoseur</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>F1,F2,F3</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>Muestreo</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>C casi seca (LAB006: GF=0.9 g/L a t=194 h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="38" customHeight="1">
-      <c r="B40" s="8" t="n">
-        <v>46295</v>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>miércoles</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Post-fin de semana: A seca esperada (t=120-146 h). Post-cambios T: F1 a 21 °C, F2 a 18 °C, F3 aún 21 °C (salta a 16 °C hoy 16:00). Descargar/respaldar datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="54" customHeight="1">
+      <c r="B41" s="7" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>lunes</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="n">
+        <v>160.5</v>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Verificar cambios T del finde + respaldo</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>Verificación</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Confirmar setpoint 18 °C en F2 (sáb 19:00); F3 cambia a 16 °C hoy 16:00 y F1 a 16 °C hoy 19:00; descargar y respaldar datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="38" customHeight="1">
+      <c r="B42" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>lunes</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
         <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="E40" s="10" t="n">
-        <v>214.5</v>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>MUESTRA -14 (t=214.5 h) + Carbodoseur</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="E42" s="10" t="n">
+        <v>166.5</v>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>MUESTRA 17 17 (t=166.5 h)</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
         <is>
           <t>F1,F2,F3</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
         <is>
           <t>Muestreo</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>Fase final de C, 4.5 h antes de su salto a 21 °C (19:00): par pre/post de Csat(T) con -15</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="22" customHeight="1">
-      <c r="B41" s="7" t="n">
-        <v>46295</v>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>miércoles</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>14:30</t>
-        </is>
-      </c>
-      <c r="E41" s="9" t="n">
-        <v>214.5</v>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>Desmontaje F1/F2 (si no se hizo el martes)</t>
-        </is>
-      </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>F1,F2</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr">
-        <is>
-          <t>Cierre</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>Limpieza de reactores liberados</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="22" customHeight="1">
-      <c r="B42" s="8" t="n">
-        <v>46295</v>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>miércoles</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="E42" s="10" t="n">
-        <v>219</v>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>Setpoint 21 °C (C)</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>Automático</t>
-        </is>
-      </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>t=219 h (réplica exacta del original)</t>
+          <t>Confirmación de sequedad de A: F1/F3 secas si GF&lt;2 g/L en -16/-17 (entonces vaciar el martes)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="38" customHeight="1">
       <c r="B43" s="7" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>lunes</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Setpoint 16 °C — F3</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>t=168 h (en el original fue inferido, sin evento registrado); lunes 16:00, con personal</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="B44" s="8" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>lunes</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="n">
+        <v>171</v>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Setpoint 16 °C — F1</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>t=171 h (réplica exacta del original)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="38" customHeight="1">
+      <c r="B45" s="7" t="n">
+        <v>46294</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>martes</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="n">
+        <v>184.5</v>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>MUESTRA 18 18 (t=184.5 h)</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Muestreo</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Confirmación A (si -17 no bastó) + cola de C. Si A confirmada: vaciar/desmontar F1 y F3 hoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="38" customHeight="1">
+      <c r="B46" s="8" t="n">
+        <v>46294</v>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>martes</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E46" s="10" t="n">
+        <v>184.5</v>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Si A confirmada seca (-16/-17): vaciar F1 y F3</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>F1,F3</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>Cierre</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Criterio: GF&lt;2 g/L en 2 muestras consecutivas (-16/-17); desmontaje de reactores liberados</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="B47" s="7" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>miércoles</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="n">
+        <v>208.5</v>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>MUESTRA 19 19 (t=208.5 h)</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Muestreo</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>C en fase final (LAB006: GF=4.7 g/L a t=170 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="38" customHeight="1">
+      <c r="B48" s="8" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>miércoles</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>MUESTRA 20 20 (t=214.5 h)</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>F1,F2,F3</t>
+        </is>
+      </c>
+      <c r="H48" s="4" t="inlineStr">
+        <is>
+          <t>Muestreo</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>C casi seca / pre-cambio T de F2 (21 °C hoy 19:00, t=219 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="B49" s="7" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>miércoles</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="n">
+        <v>219</v>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Setpoint 21 °C — F2</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Automático</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>t=219 h (réplica exacta del original)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="38" customHeight="1">
+      <c r="B50" s="8" t="n">
         <v>46296</v>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>jueves</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>08:30</t>
         </is>
       </c>
-      <c r="E43" s="9" t="n">
+      <c r="E50" s="10" t="n">
         <v>232.5</v>
       </c>
-      <c r="F43" s="3" t="inlineStr">
-        <is>
-          <t>MUESTRA -15 (condicional, solo LAB021) + Carbodoseur</t>
-        </is>
-      </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>MUESTRA -21 (condicional, solo F2) + Carbodoseur</t>
+        </is>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>Muestreo</t>
         </is>
       </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>Solo si GF(-14) &gt; 2 g/L</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="38" customHeight="1">
-      <c r="B44" s="8" t="n">
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>Solo si GF(-20) &gt; 2 g/L; luego vaciado de F2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="38" customHeight="1">
+      <c r="B51" s="7" t="n">
         <v>46296</v>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>jueves</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>09:30</t>
         </is>
       </c>
-      <c r="E44" s="10" t="n">
+      <c r="E51" s="9" t="n">
         <v>233.5</v>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F51" s="3" t="inlineStr">
         <is>
           <t>Cierre de campaña</t>
         </is>
       </c>
-      <c r="G44" s="4" t="inlineStr">
+      <c r="G51" s="3" t="inlineStr">
         <is>
           <t>F1,F2,F3</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
+      <c r="H51" s="3" t="inlineStr">
         <is>
           <t>Cierre</t>
         </is>
       </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>Desmontaje F3, descarga y respaldo final de datos, limpieza del laboratorio</t>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Vaciado/desmontaje de F2, descarga y respaldo final de datos, limpieza del laboratorio</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2424,9 +2695,9 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="46" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
@@ -2503,7 +2774,7 @@
       <c r="B5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="13" t="n">
         <v>46286.64583333334</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2529,7 +2800,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>Y15 + Alcolyzer + densidad + Brix + T mosto + DO (sin Oculyze)</t>
+          <t>Y15 + Alcolyzer + densidad + Brix + T mosto + DO (sin Oculyze; sale del contenedor de mosto)</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -2540,7 +2811,7 @@
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>[Carbo: IC del pool pre-inóculo (baseline de desgasificación)] Pre-inóculo (muestra del mosto antes de inocular): cierra la deuda de E0/YAN0 y da la IC del pool de CO2 disuelto (≠0)</t>
+          <t>[Carbo: IC del pool pre-inóculo (sale del contenedor; no consume volumen de reactores)] Pre-inóculo: cierra la deuda de E0/YAN0 y da la IC del pool de CO2 disuelto (≠0). No consume volumen de los reactores</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2819,7 @@
       <c r="B6" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <v>46286.67361111111</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2589,15 +2860,15 @@
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>[Carbo: IC del pool en t0 (≠0) + precisión de método (par PI/t0)] Muestra t=0. Par ancla PI/t0 (40 min): excepción documentada a la separación mínima; duplica la IC del pool y estima la precisión del Carbodoseur</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="102" customHeight="1">
+          <t>[Carbo: IC del pool en t0 (≠0) + precisión de método (par PI/t0)] Muestra t=0. Par ancla PI/t0 (40 min): excepción documentada a la separación mínima; YAN de t0 resuelve si el pulso 1 entra o no en la química; X0 por Oculyze</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
       <c r="B7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="11" t="n">
+      <c r="C7" s="13" t="n">
         <v>46287.35416666666</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -2638,16 +2909,16 @@
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>[Carbo: onset: acumulación vs emisión temprana (threshold vs continuous)] Fase de latencia/adaptación (CO2 detectable desde ~8-10 h). Ventana de onset: discrimina acumulación previa (threshold) vs emisión temprana (continuous)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="118" customHeight="1">
+          <t>[Carbo: trayectoria del pool pre-onset (16.5 h)] Pre-onset. Inicio de la trayectoria del pool del martes (16.5 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
       <c r="B8" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="12" t="n">
-        <v>46287.48958333334</v>
+      <c r="C8" s="14" t="n">
+        <v>46287.46875</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -2655,26 +2926,26 @@
         </is>
       </c>
       <c r="E8" s="10" t="n">
-        <v>19.75</v>
+        <v>19.25</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>LAB019-02B</t>
+          <t>LAB019-03</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>LAB020-02B</t>
+          <t>LAB020-03</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>LAB021-02B</t>
+          <t>LAB021-03</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Carbodoseur + densidad + Brix + DO (mini-muestreo: sin Y15/Oculyze/Alcolyzer)</t>
+          <t>Carbodoseur (si aplica) + densidad + Brix + DO (mini: sin Y15/Oculyze/Alcolyzer)</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
@@ -2683,19 +2954,19 @@
         </is>
       </c>
       <c r="K8" s="10" t="n">
-        <v>3.25</v>
+        <v>2.75</v>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>[Carbo: trayectoria del pool pre-onset: punto intermedio del martes (16.5/19.75/22.5 h)] Punto intermedio de la trayectoria del pool pre-onset: día martes queda 16.5 / 19.75 / 22.5 h. ~15-20 min; no interfiere con el almuerzo ni la visita de las 14:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="38" customHeight="1">
+          <t>[Carbo: trayectoria del pool pre-onset (19.25 h)] Mini-muestreo (~15-20 min): trayectoria del pool pre-onset (19.25 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
       <c r="B9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="13" t="n">
         <v>46287.60416666666</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -2708,17 +2979,17 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>LAB019-03</t>
+          <t>LAB019-04</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>LAB020-03</t>
+          <t>LAB020-04</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>LAB021-03</t>
+          <t>LAB021-04</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -2728,73 +2999,73 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="K9" s="9" t="n">
-        <v>2.75</v>
+        <v>3.25</v>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Inicio de fase exponencial</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="38" customHeight="1">
+          <t>[Carbo: borde del onset esperado de A (22.5 h)] Borde del onset esperado de A (referencias: 24-30 h según loggers de abril; 22-24 h en LAB016-018 a 20 °C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="86" customHeight="1">
       <c r="B10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="12" t="n">
-        <v>46288.35416666666</v>
+      <c r="C10" s="14" t="n">
+        <v>46287.69444444445</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>martes</t>
         </is>
       </c>
       <c r="E10" s="10" t="n">
-        <v>40.5</v>
+        <v>24.67</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>LAB019-04</t>
+          <t>LAB019-05</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>LAB020-04</t>
+          <t>LAB020-05</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>LAB021-04</t>
+          <t>LAB021-05</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+          <t>Carbodoseur (si aplica) + densidad + Brix + DO (mini: sin Y15/Oculyze/Alcolyzer)</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="K10" s="10" t="n">
-        <v>18</v>
+        <v>2.17</v>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Crecimiento exponencial; previo al pulso 2 de A (mié 19:00)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="102" customHeight="1">
+          <t>[Carbo: en/frontera del onset de A (24.7 h): discrimina threshold vs continuous] En/frontera del onset de A (~24.7 h): el punto que discrimina acumulación previa (threshold) vs emisión temprana (continuous)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
       <c r="B11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>46288.60416666666</v>
+      <c r="C11" s="13" t="n">
+        <v>46288.35416666666</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -2802,21 +3073,21 @@
         </is>
       </c>
       <c r="E11" s="9" t="n">
-        <v>46.5</v>
+        <v>40.5</v>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>LAB019-05</t>
+          <t>LAB019-06</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>LAB020-05</t>
+          <t>LAB020-06</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>LAB021-05</t>
+          <t>LAB021-06</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
@@ -2830,91 +3101,91 @@
         </is>
       </c>
       <c r="K11" s="9" t="n">
-        <v>6</v>
+        <v>15.83</v>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>[Carbo: meseta exponencial: nivel del pool vs Csat (pre-pulso A)] Última muestra antes del pulso 2 de A (19:00). Meseta exponencial: nivel del pool vs Csat. Contingencia: densidad esperada ~1044 g/L (LAB004 t=50 h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="70" customHeight="1">
+          <t>[Carbo: meseta exponencial: nivel del pool vs Csat (40.5 h)] Meseta exponencial: nivel del pool vs Csat</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
       <c r="B12" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="C12" s="12" t="n">
-        <v>46289.35416666666</v>
+      <c r="C12" s="14" t="n">
+        <v>46288.46875</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
-        <v>64.5</v>
+        <v>43.25</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>LAB019-06</t>
+          <t>LAB019-07</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>LAB020-06</t>
+          <t>LAB020-07</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>LAB021-06</t>
+          <t>LAB021-07</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+          <t>Carbodoseur (si aplica) + densidad + Brix + DO (mini: sin Y15/Oculyze/Alcolyzer)</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K12" s="10" t="n">
-        <v>18</v>
+        <v>2.75</v>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>[Carbo: respuesta del pool 13.5 h post-pulso A] 13.5 h post-pulso A: respuesta del pool al pulso. Verificar en el log que la bomba ejecutó el pulso</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="54" customHeight="1">
+          <t>Mini-muestreo de densidad (vigilar cruce de 1040 para los pulsos de la tarde)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="118" customHeight="1">
       <c r="B13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="11" t="n">
-        <v>46289.60416666666</v>
+      <c r="C13" s="13" t="n">
+        <v>46288.60416666666</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="E13" s="9" t="n">
-        <v>70.5</v>
+        <v>46.5</v>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>LAB019-07</t>
+          <t>LAB019-08</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>LAB020-07</t>
+          <t>LAB020-08</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>LAB021-07</t>
+          <t>LAB021-08</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -2924,51 +3195,51 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="K13" s="9" t="n">
-        <v>6</v>
+        <v>3.25</v>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>Última muestra antes del pulso 2 de C (jue 19:00). Contingencia: densidad esperada ~1040 g/L (LAB006 t=74 h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="38" customHeight="1">
+          <t>[Carbo: pre-pulso 2 de F3 (48 h) y F1 (51 h): nivel del pool (46.5 h)] Pre-pulso 2: F3 pulsa a las 16:00 (t=48) y F1 a las 19:00 (t=51). Contingencia densidad F1: esperada ~1044 g/L (LAB004 t=50); si ≥1052 reprogramar a jue 08:30; si ≤1036 adelantar a mié 18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="54" customHeight="1">
       <c r="B14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="C14" s="12" t="n">
-        <v>46290.35416666666</v>
+      <c r="C14" s="14" t="n">
+        <v>46288.69444444445</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="E14" s="10" t="n">
-        <v>88.5</v>
+        <v>48.67</v>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>LAB019-08</t>
+          <t>LAB019-09</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>LAB020-08</t>
+          <t>LAB020-09</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>LAB021-08</t>
+          <t>LAB021-09</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+          <t>Carbodoseur (si aplica) + densidad + Brix + DO (mini: sin Y15/Oculyze/Alcolyzer)</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
@@ -2977,11 +3248,11 @@
         </is>
       </c>
       <c r="K14" s="10" t="n">
-        <v>18</v>
+        <v>2.17</v>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>13.5 h post-pulso C; cierre de semana (salida viernes 12:30)</t>
+          <t>2.7 h post-pulso de F3 / pre-pulso de F1 (19:00): contraste entre fermentadores en la misma visita</t>
         </is>
       </c>
     </row>
@@ -2989,30 +3260,30 @@
       <c r="B15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>46293.35416666666</v>
+      <c r="C15" s="13" t="n">
+        <v>46289.35416666666</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="E15" s="9" t="n">
-        <v>160.5</v>
+        <v>64.5</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>LAB019-09</t>
+          <t>LAB019-10</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>LAB020-09</t>
+          <t>LAB020-10</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>LAB021-09</t>
+          <t>LAB021-10</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -3026,47 +3297,47 @@
         </is>
       </c>
       <c r="K15" s="9" t="n">
-        <v>72</v>
+        <v>15.83</v>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>[Carbo: post-cambios T (A 21 °C, C 18 °C): valida Csat(T)] Post-fin de semana: A seca esperada (t=122-146 h). Post-cambios T (A 21 °C, C 18 °C): valida Csat(T). Descargar/respaldar datos</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="54" customHeight="1">
+          <t>[Carbo: post-pulso de F1/F3 (13.5-16.5 h después) (64.5 h)] Post-pulso: F1 a 13.5 h y F3 a 16.5 h del suyo; F2 pre-pulso (75 h = jue 19:00). Verificar logs de bomba del miércoles</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
       <c r="B16" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C16" s="12" t="n">
-        <v>46293.60416666666</v>
+      <c r="C16" s="14" t="n">
+        <v>46289.46875</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="E16" s="10" t="n">
-        <v>166.5</v>
+        <v>67.25</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>LAB019-10</t>
+          <t>LAB019-11</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>LAB020-10</t>
+          <t>LAB020-11</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>LAB021-10</t>
+          <t>LAB021-11</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+          <t>Carbodoseur (si aplica) + densidad + Brix + DO (mini: sin Y15/Oculyze/Alcolyzer)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -3075,42 +3346,42 @@
         </is>
       </c>
       <c r="K16" s="10" t="n">
-        <v>6</v>
+        <v>2.75</v>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Confirmación de sequedad A (GF&lt;2 g/L en 2 muestras seguidas da por terminados LAB019/020)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="38" customHeight="1">
+          <t>Mini-muestreo de densidad (cruce de 1040 de F2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="86" customHeight="1">
       <c r="B17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>46294.35416666666</v>
+      <c r="C17" s="13" t="n">
+        <v>46289.60416666666</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>martes</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="E17" s="9" t="n">
-        <v>184.5</v>
+        <v>70.5</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>LAB019-11</t>
+          <t>LAB019-12</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>LAB020-11</t>
+          <t>LAB020-12</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>LAB021-11</t>
+          <t>LAB021-12</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -3124,11 +3395,11 @@
         </is>
       </c>
       <c r="K17" s="9" t="n">
-        <v>18</v>
+        <v>3.25</v>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>Muestra final de A (condicional); C en fase final</t>
+          <t>Última muestra antes del pulso 2 de F2 (19:00). Contingencia densidad: esperada ~1040 g/L (LAB006 t=74); si ≥1048 reprogramar a vie 08:30; si ≤1032 adelantar a jue 18:00</t>
         </is>
       </c>
     </row>
@@ -3136,35 +3407,35 @@
       <c r="B18" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C18" s="12" t="n">
-        <v>46294.60416666666</v>
+      <c r="C18" s="14" t="n">
+        <v>46289.69444444445</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>martes</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="E18" s="10" t="n">
-        <v>190.5</v>
+        <v>72.67</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>LAB019-12</t>
+          <t>LAB019-13</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>LAB020-12</t>
+          <t>LAB020-13</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>LAB021-12</t>
+          <t>LAB021-13</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+          <t>Carbodoseur (si aplica) + densidad + Brix + DO (mini: sin Y15/Oculyze/Alcolyzer)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -3173,42 +3444,42 @@
         </is>
       </c>
       <c r="K18" s="10" t="n">
-        <v>6</v>
+        <v>2.17</v>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Cercanía a sequedad de C (LAB006: GF=4.7 g/L a t=170 h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="38" customHeight="1">
+          <t>2.7 h pre-pulso de F2 (19:00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="86" customHeight="1">
       <c r="B19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="C19" s="11" t="n">
-        <v>46295.35416666666</v>
+      <c r="C19" s="13" t="n">
+        <v>46290.35416666666</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="E19" s="9" t="n">
-        <v>208.5</v>
+        <v>88.5</v>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>LAB019-13</t>
+          <t>LAB019-14</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>LAB020-13</t>
+          <t>LAB020-14</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>LAB021-13</t>
+          <t>LAB021-14</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
@@ -3218,113 +3489,358 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>SÍ</t>
         </is>
       </c>
       <c r="K19" s="9" t="n">
-        <v>18</v>
+        <v>15.83</v>
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>C casi seca (LAB006: GF=0.9 g/L a t=194 h)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="70" customHeight="1">
+          <t>[Carbo: post-pulso de F2 (13.5 h) (88.5 h)] Post-pulso de F2 (13.5 h) + A tardía. Verificar log del pulso de F2 y del cambio T de F3 (vie 16:00); F1 cambia a 21 °C hoy 19:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
       <c r="B20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="C20" s="12" t="n">
-        <v>46295.60416666666</v>
+      <c r="C20" s="14" t="n">
+        <v>46290.45833333334</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="E20" s="10" t="n">
-        <v>214.5</v>
+        <v>91</v>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>LAB019-14</t>
+          <t>LAB019-15</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>LAB020-14</t>
+          <t>LAB020-15</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>LAB021-14</t>
+          <t>LAB021-15</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+          <t>Carbodoseur (si aplica) + densidad + Brix + DO (mini: sin Y15/Oculyze/Alcolyzer)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K20" s="10" t="n">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>[Carbo: fase final de C, antes de su salto a 21 °C] Fase final de C, 4.5 h antes de su salto a 21 °C (19:00): par pre/post de Csat(T) con -15</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="86" customHeight="1">
+          <t>Última del día antes del cambio T de F1 (19:00); cierre de semana (salida 12:30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="102" customHeight="1">
       <c r="B21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="C21" s="11" t="n">
+      <c r="C21" s="13" t="n">
+        <v>46293.35416666666</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>lunes</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>160.5</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>LAB019-16</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>LAB020-16</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>LAB021-16</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>[Carbo: post-cambios T del finde: F1 21 °C, F2 18 °C, F3 21 °C -&gt; valida Csat(T) (160.5 h)] Post-fin de semana: A seca esperada (t=120-146 h). Post-cambios T: F1 a 21 °C, F2 a 18 °C, F3 aún 21 °C (salta a 16 °C hoy 16:00). Descargar/respaldar datos</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1">
+      <c r="B22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>46293.60416666666</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>lunes</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>166.5</v>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>LAB019-17</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>LAB020-17</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>LAB021-17</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Confirmación de sequedad de A: F1/F3 secas si GF&lt;2 g/L en -16/-17 (entonces vaciar el martes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="B23" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C23" s="13" t="n">
+        <v>46294.35416666666</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>martes</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n">
+        <v>184.5</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>LAB019-18</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>LAB020-18</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>LAB021-18</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Confirmación A (si -17 no bastó) + cola de C. Si A confirmada: vaciar/desmontar F1 y F3 hoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="B24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>46295.35416666666</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>miércoles</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>208.5</v>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>LAB019-19</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>LAB020-19</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>LAB021-19</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>C en fase final (LAB006: GF=4.7 g/L a t=170 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="B25" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C25" s="13" t="n">
+        <v>46295.60416666666</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>miércoles</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>214.5</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>LAB019-20</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>LAB020-20</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>LAB021-20</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>C casi seca / pre-cambio T de F2 (21 °C hoy 19:00, t=219 h)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="86" customHeight="1">
+      <c r="B26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="C26" s="14" t="n">
         <v>46296.35416666666</v>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>jueves</t>
         </is>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E26" s="10" t="n">
         <v>232.5</v>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>LAB020-21</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>LAB021-15</t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Y15 + Alcolyzer + Oculyze + densidad + Brix + DO</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>SÍ (cond.)</t>
         </is>
       </c>
-      <c r="K21" s="9" t="n">
+      <c r="K26" s="10" t="n">
         <v>18</v>
       </c>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>[Carbo: post-salto T de C (13 h): cierre del par térmico] Solo LAB021 y solo si GF(-14) &gt; 2 g/L; 13 h después del salto a 21 °C de C: cierre del par térmico. Luego desmontaje y cierre de campaña</t>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>[Carbo: post-salto T de F2 (13 h): cierre del par térmico (232.5 h)] CONDICIONAL: solo F2 y solo si GF(-20) &gt; 2 g/L; 13 h después del salto a 21 °C. Luego vaciado de F2 y cierre de campaña</t>
         </is>
       </c>
     </row>
@@ -3343,12 +3859,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
@@ -3407,7 +3923,7 @@
     <row r="6" ht="38" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>LAB019/020 (A)</t>
+          <t>LAB019 (A, de LAB004)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -3421,19 +3937,19 @@
       <c r="E6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="13" t="n">
         <v>46286.66666666666</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Setpoint inicial; carga del mosto ya equilibrado el lunes</t>
+          <t>Setpoint inicial; mosto cargado ya equilibrado</t>
         </is>
       </c>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>LAB019/020 (A)</t>
+          <t>LAB019 (A, de LAB004)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -3447,7 +3963,7 @@
       <c r="E7" s="10" t="n">
         <v>99</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="14" t="n">
         <v>46290.79166666666</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -3459,7 +3975,7 @@
     <row r="8" ht="38" customHeight="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>LAB019/020 (A)</t>
+          <t>LAB019 (A, de LAB004)</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -3473,7 +3989,7 @@
       <c r="E8" s="9" t="n">
         <v>171</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="13" t="n">
         <v>46293.79166666666</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3485,7 +4001,7 @@
     <row r="9" ht="38" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>LAB021 (C)</t>
+          <t>LAB020 (C, de LAB006)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -3499,7 +4015,7 @@
       <c r="E9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="14" t="n">
         <v>46286.66666666666</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -3511,7 +4027,7 @@
     <row r="10" ht="38" customHeight="1">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>LAB021 (C)</t>
+          <t>LAB020 (C, de LAB006)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -3525,7 +4041,7 @@
       <c r="E10" s="9" t="n">
         <v>123</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="13" t="n">
         <v>46291.79166666666</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
@@ -3537,7 +4053,7 @@
     <row r="11" ht="38" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>LAB021 (C)</t>
+          <t>LAB020 (C, de LAB006)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -3551,7 +4067,7 @@
       <c r="E11" s="10" t="n">
         <v>219</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="14" t="n">
         <v>46295.79166666666</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -3560,145 +4076,256 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1"/>
-    <row r="13" ht="24" customHeight="1">
-      <c r="B13" s="5" t="inlineStr">
+    <row r="12" ht="38" customHeight="1">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>LAB021 (A, de LAB009)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Fase 1</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>46286.66666666666</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Setpoint inicial</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>LAB021 (A, de LAB009)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Fase 2</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>96</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>46290.66666666666</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Automático (viernes 25/09 16:00, con personal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>LAB021 (A, de LAB009)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Fase 3</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>46293.66666666666</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Automático (lunes 28/09 16:00; en el original fue inferido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1"/>
+    <row r="16" ht="24" customHeight="1">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Pulsos nutricionales (automatizados por bomba peristáltica)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="2" t="inlineStr">
+    <row r="17" ht="28" customHeight="1">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Evento</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Reactores</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Producto y dosis</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>t [h]</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Fecha-hora</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Vía</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Verificación / contingencia</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="38" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
+    <row r="18" ht="38" customHeight="1">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Pulso 1 (con la inoculación)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>F1,F2,F3</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Springferm Xtrem 1.00 g + FDA 0.40 g por reactor (va dentro del inóculo)</t>
         </is>
       </c>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="11" t="n">
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="13" t="n">
         <v>46286.66319444445</v>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Bomba peristáltica</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>50% del suplemento total; igual en A y C (regla original)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="70" customHeight="1">
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Pulso 2 — condición A</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>F1,F2 (LAB019/020)</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
+    <row r="19" ht="86" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Pulso 2 — F3 (A, de LAB009)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>F3 (LAB021)</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Springferm Xtrem 1.00 g + FDA 0.40 g</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>46288.66666666666</v>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>Bomba peristáltica</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>Original sin registro en workbook: t=48 h según ICS (19/04); densidad cruzó 1040 ~t=44 h. Contingencia: si densidad(-07, mié 11:15) ≥ 1052 g/L, reprogramar a mié 19:00; si ≤1036, adelantar a mié 14:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="70" customHeight="1">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Pulso 2 — F1 (A, de LAB004)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>F1 (LAB019)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Springferm Xtrem 1.00 g + FDA 0.40 g por reactor</t>
         </is>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E20" s="9" t="n">
         <v>51</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F20" s="13" t="n">
         <v>46288.79166666666</v>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Bomba peristáltica</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Original: al cruzar densidad 1040 (LAB004/005 t=51 h). Contingencia: si densidad(-05, mié 14:30) ≥ 1052 g/L, reprogramar a jue 08:30; si ≤ 1036, adelantar a mié 16:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="70" customHeight="1">
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Pulso 2 — condición C</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>F3 (LAB021)</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Original: al cruzar densidad 1040 (LAB004 t=51 h). Contingencia: si densidad(-08, mié 14:30) ≥ 1052 g/L, reprogramar a jue 08:30; si ≤1036, adelantar a mié 18:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="70" customHeight="1">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Pulso 2 — F2 (C, de LAB006)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>F2 (LAB020)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Springferm Xtrem 1.00 g + FDA 0.40 g</t>
         </is>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E21" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="F21" s="14" t="n">
         <v>46289.79166666666</v>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Bomba peristáltica</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Original: densidad 1040 a t=75 h (LAB006). Contingencia: si densidad(-07, jue 14:30) ≥ 1048 g/L, reprogramar a vie 08:30; si ≤ 1032, adelantar a jue 16:30</t>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Original: densidad 1040 a t=75 h (LAB006). Contingencia: si densidad(-12, jue 14:30) ≥ 1048 g/L, reprogramar a vie 08:30; si ≤1032, adelantar a jue 18:00</t>
         </is>
       </c>
     </row>
@@ -3716,7 +4343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3745,7 +4372,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1">
+    <row r="5" ht="38" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Horario lun-jue</t>
@@ -3753,11 +4380,11 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Trabajo 8:00-17:30. Visitas de muestreo 08:30 y 14:30; cada visita demora ~1.5-2 h de procesamiento (08:30→~10:30; 14:30→~16:30, con margen antes de la limpieza de 17:00). Almuerzo 13:00-14:30</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="38" customHeight="1">
+          <t>Trabajo 8:00-17:30. Visitas completas 08:30 y 14:30 (~1.5-2 h de proceso cada una) + mini-muestreos 11:15 y 16:40 (~15-20 min). Almuerzo 13:00-14:30; limpieza desde 17:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Horario viernes</t>
@@ -3765,7 +4392,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Trabajo 8:00-12:30. Visita única 08:30 (~2 h de proceso, listo ~10:30); limpieza 12:00-12:30</t>
+          <t>Trabajo 8:00-12:30. Visita completa 08:30 (~2 h) + mini 11:00; limpieza 12:00-12:30</t>
         </is>
       </c>
     </row>
@@ -3777,7 +4404,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Sin personal (sáb 26 y dom 27/09). Solo logging continuo de CO2/T y eventos automáticos ya programados</t>
+          <t>Sin personal (sáb 26 y dom 27/09). Solo logging continuo de CO2/T y eventos automáticos ya programados (setpoint F2 18 °C sáb 19:00)</t>
         </is>
       </c>
     </row>
@@ -3789,7 +4416,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Mínimo 2 h (piso absoluto 1.5 h). Visitas completas a 6 h intra-día (08:30/14:30) y 18 h entre días; el mini -02B queda a 3.25/2.75 h de sus vecinas (solo Carbodoseur + densidad, sin carga de Y15); menos muestras y mejor separadas</t>
+          <t>Mínimo 2 h (piso absoluto 1.5 h). Grid mar-jue: 08:30 / 11:15 / 14:30 / 16:40 (2.2-3.3 h entre muestras; los minis son livianos, sin Y15). Entre días 15.8-18 h. Excepción PI/t0 (40 min)</t>
         </is>
       </c>
     </row>
@@ -3801,11 +4428,11 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>El par PI (15:30) y t0 (16:10) del lunes está separado 40 min: par ancla pre/post inoculación recomendado por las auditorías; además duplica la IC del pool de CO2 y estima la precisión del Carbodoseur</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="70" customHeight="1">
+          <t>El par PI (15:30) y t0 (16:10) del lunes está separado 40 min: par ancla pre/post inoculación; el YAN de t0 resuelve si el pulso 1 entra en la química; el Oculyze de t0 da el X0 real</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Procesamiento por visita</t>
@@ -3813,7 +4440,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>~1.5-2 h: 3 fermentadores × (Y15 + Alcolyzer + Oculyze + Brix + densidad + DO + Carbodoseur cuando aplica). Por eso la visita de tarde parte a las 14:30 y no a las 15:00. El mini-muestreo -02B (mar 11:45) es solo Carbodoseur + densidad/Brix/DO: ~15-20 min, sin Y15/Oculyze/Alcolyzer</t>
+          <t>Visita completa ~1.5-2 h: 3 fermentadores × (Y15 + Alcolyzer + Oculyze + Brix + densidad + DO + Carbodoseur cuando aplica). Mini-muestreo ~15-20 min (solo instrumental)</t>
         </is>
       </c>
     </row>
@@ -3825,7 +4452,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Tomar SIEMPRE la primera alícuota, directo del puerto y sin burbujear. Anotar en la planilla de registro: volumen remanente (mL) y T de medición; el CO2 disuelto se completa después con la tabla digitalizada. ~100 mL por lectura</t>
+          <t>Tomar SIEMPRE la primera alícuota, directo del puerto y sin burbujear. Anotar en la planilla de registro: volumen remanente (mL) y T de medición; el CO2 disuelto se completa después con la tabla digitalizada. ~100 mL por lectura (la alícuota SE DEVUELVE al reactor; «Vol. rem.» es solo control operativo)</t>
         </is>
       </c>
     </row>
@@ -3837,7 +4464,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Fijos: PI, -01, -02, -02B, -05, -06, -09, -14. Condicional: -15 (si se toma). Motivo: pool de CO2 disuelto observable — IC real (≠0, hoy el modelo parte en 0), trayectoria pre/post onset para discriminar threshold vs continuous release y validación de Csat(T) en los cambios de setpoint</t>
+          <t>11 fijas: PI, -01, -02 a -05 (mar: trayectoria del onset 16.5/19.25/22.5/24.7 h), -06 y -08 (mié: meseta y pre-pulso), -10 (jue: post-pulso F1/F3), -14 (vie: post-pulso F2), -16 (lun 28: post-cambios T). Condicional: -21. PI sale del contenedor (no consume volumen de reactores)</t>
         </is>
       </c>
     </row>
@@ -3849,7 +4476,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2 L iniciales por reactor. Presupuesto estimado: ~0.8-0.9 L de Carbodoseur (9 lecturas) + ~0.4-0.6 L de química ≈ 65-75% del batch. Registrar volumen acumulado por reactor; si el volumen se vuelve crítico, las lecturas Carbodoseur de -14/-15 son las primeras a suspender</t>
+          <t>2 L iniciales por reactor. La alícuota del Carbodoseur (~100 mL) SE DEVUELVE al reactor: no se pierde; «Vol. remanente» es solo control operativo. Pérdidas no retornables por reactor: Alcolyzer 50 mL por muestra (F1/F3: mar-mié-jue ≈3 muestras = 150 mL; F2 ≈5 muestras = 250 mL), Y15 1 mL + Oculyze 1 mL por visita completa y ~2 mL por visita de mangueras/operación (también en minis). Pérdida total ≈0.2 L (F1/F3) y ≈0.3 L (F2): volumen final ≈1.7-1.8 L de los 2.0 L iniciales. Registrar volumen acumulado como control</t>
         </is>
       </c>
     </row>
@@ -3873,7 +4500,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>LAB019/020 terminan cuando GF &lt; 2 g/L en 2 muestras consecutivas (esperado -09/-10 del lunes 28/09); luego vaciado y desmontaje</t>
+          <t>F1/F3 (LAB019/021) terminan cuando GF &lt; 2 g/L en 2 muestras consecutivas (esperado -16/-17 del lunes 28/09); vaciar/desmontar el martes 29</t>
         </is>
       </c>
     </row>
@@ -3885,7 +4512,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>LAB021 termina cuando GF &lt; 2 g/L en 2 muestras consecutivas (esperado -13/-14 del miércoles 30/09); -15 (jue 01/10) solo si GF(-14) &gt; 2 g/L</t>
+          <t>F2 (LAB020) termina cuando GF &lt; 2 g/L en 2 muestras consecutivas (esperado -19/-20 del miércoles 30/09); -21 (jue 01/10) solo si GF(-20) &gt; 2 g/L</t>
         </is>
       </c>
     </row>
@@ -3901,7 +4528,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="38" customHeight="1">
+    <row r="18" ht="70" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Contingencia fugas CO2</t>
@@ -3909,7 +4536,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Verificar conexiones el lunes a.m. y revisar trazas diariamente: caída a cero o baseline asimétrico F1 vs F2/F3 son señales de fuga (ref. auditoría LAB001-018)</t>
+          <t>Verificar conexiones el lunes a.m. y revisar trazas diariamente: durante el lag las trazas NO debieran estar en 0.000 exactos (la desorción da ~0.5-1 sccm) ni saltar de golpe; cero plano = línea sospechosa (patrón F1 de abril); baseline creciente = sospecha de fuga (patrón F2/F3 de abril)</t>
         </is>
       </c>
     </row>
@@ -3921,7 +4548,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>La sequedad de A (t=122-146 h) caerá dentro del fin de semana sin muestreo; la señal continua de CO2 (objetivo de esta réplica) cubre el intervalo. Mencionar en el análisis posterior</t>
+          <t>La sequedad de A (t=120-146 h) caerá entre el sábado 16:00 y el domingo 18:00 sin muestreo; la señal continua de CO2 (objetivo de esta réplica) cubre el intervalo. Mencionar en el análisis posterior</t>
         </is>
       </c>
     </row>
@@ -3934,6 +4561,18 @@
       <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Nombrar canales de logger LAB019/020/021 (CO2 y T) antes del lunes 16:00; registrar en el log la hora exacta del flanco de cada bomba; descargar y respaldar el lunes 28 a.m. y al cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Nota LAB009</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Réplica de LAB009: sin registro en Maestro_ensayos; pulso 2 por ICS (t=48 h) y cambio T a 16 °C a t=168 h inferido en el original; su CO2 histórico también fue excluido por QC, igual que LAB004/006 — por eso estos tres son los que más ganan con la réplica</t>
         </is>
       </c>
     </row>

</xml_diff>